<commit_message>
Add latest changes to monorepo
</commit_message>
<xml_diff>
--- a/backend/scheduler/services/resource/data/simulation/telescope_schedules.xlsx
+++ b/backend/scheduler/services/resource/data/simulation/telescope_schedules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bmiller/python/scheduler/scheduler/services/resource/data/simulation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE7F8F9F-17AF-C845-847E-856F6431E73D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78F0ACF3-54E3-DC49-9E65-BF132583218B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="3700" windowWidth="36000" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3700" windowWidth="36000" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GS" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21158" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22103" uniqueCount="39">
   <si>
     <t>Local Date</t>
   </si>
@@ -445,7 +445,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AD612"/>
+  <dimension ref="A1:AD639"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="2" max="2" width="8.6640625" customWidth="1"/>
@@ -40593,6 +40593,1896 @@
       <c r="AB612" s="2"/>
       <c r="AC612" s="2"/>
       <c r="AD612" s="2"/>
+    </row>
+    <row r="613" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A613" s="5">
+        <v>46116</v>
+      </c>
+      <c r="B613" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C613" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D613" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E613" s="2"/>
+      <c r="F613" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G613" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H613" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I613" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J613" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K613" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L613" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M613" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N613" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O613" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P613" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q613" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R613" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S613" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T613" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U613" s="2"/>
+      <c r="V613" s="2"/>
+      <c r="W613" s="2"/>
+      <c r="X613" s="2"/>
+      <c r="Y613" s="2"/>
+      <c r="Z613" s="2"/>
+      <c r="AA613" s="2"/>
+      <c r="AB613" s="2"/>
+      <c r="AC613" s="2"/>
+      <c r="AD613" s="2"/>
+    </row>
+    <row r="614" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A614" s="5">
+        <v>46117</v>
+      </c>
+      <c r="B614" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C614" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D614" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E614" s="2"/>
+      <c r="F614" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G614" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H614" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I614" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J614" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K614" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L614" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M614" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N614" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O614" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P614" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q614" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R614" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S614" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T614" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U614" s="2"/>
+      <c r="V614" s="2"/>
+      <c r="W614" s="2"/>
+      <c r="X614" s="2"/>
+      <c r="Y614" s="2"/>
+      <c r="Z614" s="2"/>
+      <c r="AA614" s="2"/>
+      <c r="AB614" s="2"/>
+      <c r="AC614" s="2"/>
+      <c r="AD614" s="2"/>
+    </row>
+    <row r="615" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A615" s="5">
+        <v>46118</v>
+      </c>
+      <c r="B615" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C615" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D615" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E615" s="2"/>
+      <c r="F615" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G615" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H615" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I615" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J615" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K615" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L615" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M615" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N615" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O615" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P615" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q615" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R615" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S615" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T615" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U615" s="2"/>
+      <c r="V615" s="2"/>
+      <c r="W615" s="2"/>
+      <c r="X615" s="2"/>
+      <c r="Y615" s="2"/>
+      <c r="Z615" s="2"/>
+      <c r="AA615" s="2"/>
+      <c r="AB615" s="2"/>
+      <c r="AC615" s="2"/>
+      <c r="AD615" s="2"/>
+    </row>
+    <row r="616" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A616" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B616" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C616" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D616" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E616" s="2"/>
+      <c r="F616" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G616" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H616" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I616" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J616" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K616" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L616" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M616" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N616" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O616" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P616" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q616" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R616" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S616" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T616" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U616" s="2"/>
+      <c r="V616" s="2"/>
+      <c r="W616" s="2"/>
+      <c r="X616" s="2"/>
+      <c r="Y616" s="2"/>
+      <c r="Z616" s="2"/>
+      <c r="AA616" s="2"/>
+      <c r="AB616" s="2"/>
+      <c r="AC616" s="2"/>
+      <c r="AD616" s="2"/>
+    </row>
+    <row r="617" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A617" s="5">
+        <v>46120</v>
+      </c>
+      <c r="B617" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C617" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D617" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E617" s="2"/>
+      <c r="F617" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G617" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H617" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I617" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J617" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K617" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L617" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M617" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N617" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O617" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P617" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q617" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R617" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S617" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T617" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U617" s="2"/>
+      <c r="V617" s="2"/>
+      <c r="W617" s="2"/>
+      <c r="X617" s="2"/>
+      <c r="Y617" s="2"/>
+      <c r="Z617" s="2"/>
+      <c r="AA617" s="2"/>
+      <c r="AB617" s="2"/>
+      <c r="AC617" s="2"/>
+      <c r="AD617" s="2"/>
+    </row>
+    <row r="618" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A618" s="5">
+        <v>46121</v>
+      </c>
+      <c r="B618" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C618" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D618" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E618" s="2"/>
+      <c r="F618" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G618" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H618" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I618" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J618" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K618" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L618" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M618" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N618" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O618" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P618" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q618" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R618" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S618" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T618" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U618" s="2"/>
+      <c r="V618" s="2"/>
+      <c r="W618" s="2"/>
+      <c r="X618" s="2"/>
+      <c r="Y618" s="2"/>
+      <c r="Z618" s="2"/>
+      <c r="AA618" s="2"/>
+      <c r="AB618" s="2"/>
+      <c r="AC618" s="2"/>
+      <c r="AD618" s="2"/>
+    </row>
+    <row r="619" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A619" s="5">
+        <v>46122</v>
+      </c>
+      <c r="B619" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C619" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D619" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E619" s="2"/>
+      <c r="F619" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G619" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H619" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I619" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J619" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K619" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L619" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M619" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N619" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O619" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P619" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q619" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R619" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S619" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T619" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U619" s="2"/>
+      <c r="V619" s="2"/>
+      <c r="W619" s="2"/>
+      <c r="X619" s="2"/>
+      <c r="Y619" s="2"/>
+      <c r="Z619" s="2"/>
+      <c r="AA619" s="2"/>
+      <c r="AB619" s="2"/>
+      <c r="AC619" s="2"/>
+      <c r="AD619" s="2"/>
+    </row>
+    <row r="620" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A620" s="5">
+        <v>46123</v>
+      </c>
+      <c r="B620" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C620" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D620" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E620" s="2"/>
+      <c r="F620" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G620" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H620" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I620" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J620" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K620" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L620" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M620" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N620" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O620" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P620" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q620" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R620" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S620" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T620" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U620" s="2"/>
+      <c r="V620" s="2"/>
+      <c r="W620" s="2"/>
+      <c r="X620" s="2"/>
+      <c r="Y620" s="2"/>
+      <c r="Z620" s="2"/>
+      <c r="AA620" s="2"/>
+      <c r="AB620" s="2"/>
+      <c r="AC620" s="2"/>
+      <c r="AD620" s="2"/>
+    </row>
+    <row r="621" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A621" s="5">
+        <v>46124</v>
+      </c>
+      <c r="B621" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C621" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D621" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E621" s="2"/>
+      <c r="F621" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G621" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H621" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I621" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J621" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K621" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L621" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M621" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N621" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O621" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P621" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q621" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R621" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S621" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T621" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U621" s="2"/>
+      <c r="V621" s="2"/>
+      <c r="W621" s="2"/>
+      <c r="X621" s="2"/>
+      <c r="Y621" s="2"/>
+      <c r="Z621" s="2"/>
+      <c r="AA621" s="2"/>
+      <c r="AB621" s="2"/>
+      <c r="AC621" s="2"/>
+      <c r="AD621" s="2"/>
+    </row>
+    <row r="622" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A622" s="5">
+        <v>46125</v>
+      </c>
+      <c r="B622" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C622" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D622" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E622" s="2"/>
+      <c r="F622" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G622" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H622" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I622" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J622" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K622" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L622" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M622" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N622" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O622" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P622" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q622" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R622" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S622" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T622" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U622" s="2"/>
+      <c r="V622" s="2"/>
+      <c r="W622" s="2"/>
+      <c r="X622" s="2"/>
+      <c r="Y622" s="2"/>
+      <c r="Z622" s="2"/>
+      <c r="AA622" s="2"/>
+      <c r="AB622" s="2"/>
+      <c r="AC622" s="2"/>
+      <c r="AD622" s="2"/>
+    </row>
+    <row r="623" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A623" s="5">
+        <v>46126</v>
+      </c>
+      <c r="B623" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C623" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D623" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E623" s="2"/>
+      <c r="F623" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G623" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H623" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I623" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J623" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K623" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L623" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M623" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N623" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O623" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P623" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q623" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R623" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S623" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T623" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U623" s="2"/>
+      <c r="V623" s="2"/>
+      <c r="W623" s="2"/>
+      <c r="X623" s="2"/>
+      <c r="Y623" s="2"/>
+      <c r="Z623" s="2"/>
+      <c r="AA623" s="2"/>
+      <c r="AB623" s="2"/>
+      <c r="AC623" s="2"/>
+      <c r="AD623" s="2"/>
+    </row>
+    <row r="624" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A624" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B624" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C624" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D624" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E624" s="2"/>
+      <c r="F624" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G624" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H624" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I624" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J624" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K624" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L624" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M624" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N624" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O624" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P624" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q624" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R624" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S624" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T624" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U624" s="2"/>
+      <c r="V624" s="2"/>
+      <c r="W624" s="2"/>
+      <c r="X624" s="2"/>
+      <c r="Y624" s="2"/>
+      <c r="Z624" s="2"/>
+      <c r="AA624" s="2"/>
+      <c r="AB624" s="2"/>
+      <c r="AC624" s="2"/>
+      <c r="AD624" s="2"/>
+    </row>
+    <row r="625" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A625" s="5">
+        <v>46128</v>
+      </c>
+      <c r="B625" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C625" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D625" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E625" s="2"/>
+      <c r="F625" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G625" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H625" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I625" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J625" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K625" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L625" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M625" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N625" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O625" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P625" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q625" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R625" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S625" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T625" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U625" s="2"/>
+      <c r="V625" s="2"/>
+      <c r="W625" s="2"/>
+      <c r="X625" s="2"/>
+      <c r="Y625" s="2"/>
+      <c r="Z625" s="2"/>
+      <c r="AA625" s="2"/>
+      <c r="AB625" s="2"/>
+      <c r="AC625" s="2"/>
+      <c r="AD625" s="2"/>
+    </row>
+    <row r="626" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A626" s="5">
+        <v>46129</v>
+      </c>
+      <c r="B626" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C626" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D626" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E626" s="2"/>
+      <c r="F626" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G626" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H626" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I626" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J626" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K626" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L626" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M626" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N626" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O626" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P626" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q626" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R626" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S626" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T626" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U626" s="2"/>
+      <c r="V626" s="2"/>
+      <c r="W626" s="2"/>
+      <c r="X626" s="2"/>
+      <c r="Y626" s="2"/>
+      <c r="Z626" s="2"/>
+      <c r="AA626" s="2"/>
+      <c r="AB626" s="2"/>
+      <c r="AC626" s="2"/>
+      <c r="AD626" s="2"/>
+    </row>
+    <row r="627" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A627" s="5">
+        <v>46130</v>
+      </c>
+      <c r="B627" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C627" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D627" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E627" s="2"/>
+      <c r="F627" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G627" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H627" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I627" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J627" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K627" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L627" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M627" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N627" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O627" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P627" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q627" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R627" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S627" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T627" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U627" s="2"/>
+      <c r="V627" s="2"/>
+      <c r="W627" s="2"/>
+      <c r="X627" s="2"/>
+      <c r="Y627" s="2"/>
+      <c r="Z627" s="2"/>
+      <c r="AA627" s="2"/>
+      <c r="AB627" s="2"/>
+      <c r="AC627" s="2"/>
+      <c r="AD627" s="2"/>
+    </row>
+    <row r="628" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A628" s="5">
+        <v>46131</v>
+      </c>
+      <c r="B628" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C628" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D628" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E628" s="2"/>
+      <c r="F628" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G628" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H628" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I628" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J628" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K628" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L628" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M628" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N628" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O628" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P628" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q628" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R628" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S628" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T628" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U628" s="2"/>
+      <c r="V628" s="2"/>
+      <c r="W628" s="2"/>
+      <c r="X628" s="2"/>
+      <c r="Y628" s="2"/>
+      <c r="Z628" s="2"/>
+      <c r="AA628" s="2"/>
+      <c r="AB628" s="2"/>
+      <c r="AC628" s="2"/>
+      <c r="AD628" s="2"/>
+    </row>
+    <row r="629" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A629" s="5">
+        <v>46132</v>
+      </c>
+      <c r="B629" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C629" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D629" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E629" s="2"/>
+      <c r="F629" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G629" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H629" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I629" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J629" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K629" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L629" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M629" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N629" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O629" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P629" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q629" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R629" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S629" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T629" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U629" s="2"/>
+      <c r="V629" s="2"/>
+      <c r="W629" s="2"/>
+      <c r="X629" s="2"/>
+      <c r="Y629" s="2"/>
+      <c r="Z629" s="2"/>
+      <c r="AA629" s="2"/>
+      <c r="AB629" s="2"/>
+      <c r="AC629" s="2"/>
+      <c r="AD629" s="2"/>
+    </row>
+    <row r="630" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A630" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B630" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C630" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D630" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E630" s="2"/>
+      <c r="F630" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G630" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H630" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I630" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J630" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K630" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L630" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M630" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N630" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O630" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P630" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q630" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R630" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S630" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T630" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U630" s="2"/>
+      <c r="V630" s="2"/>
+      <c r="W630" s="2"/>
+      <c r="X630" s="2"/>
+      <c r="Y630" s="2"/>
+      <c r="Z630" s="2"/>
+      <c r="AA630" s="2"/>
+      <c r="AB630" s="2"/>
+      <c r="AC630" s="2"/>
+      <c r="AD630" s="2"/>
+    </row>
+    <row r="631" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A631" s="5">
+        <v>46134</v>
+      </c>
+      <c r="B631" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C631" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D631" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E631" s="2"/>
+      <c r="F631" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G631" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H631" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I631" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J631" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K631" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L631" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M631" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N631" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O631" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P631" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q631" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R631" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S631" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T631" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U631" s="2"/>
+      <c r="V631" s="2"/>
+      <c r="W631" s="2"/>
+      <c r="X631" s="2"/>
+      <c r="Y631" s="2"/>
+      <c r="Z631" s="2"/>
+      <c r="AA631" s="2"/>
+      <c r="AB631" s="2"/>
+      <c r="AC631" s="2"/>
+      <c r="AD631" s="2"/>
+    </row>
+    <row r="632" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A632" s="5">
+        <v>46135</v>
+      </c>
+      <c r="B632" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C632" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D632" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E632" s="2"/>
+      <c r="F632" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G632" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H632" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I632" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J632" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K632" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L632" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M632" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N632" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O632" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P632" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q632" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R632" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S632" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T632" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U632" s="2"/>
+      <c r="V632" s="2"/>
+      <c r="W632" s="2"/>
+      <c r="X632" s="2"/>
+      <c r="Y632" s="2"/>
+      <c r="Z632" s="2"/>
+      <c r="AA632" s="2"/>
+      <c r="AB632" s="2"/>
+      <c r="AC632" s="2"/>
+      <c r="AD632" s="2"/>
+    </row>
+    <row r="633" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A633" s="5">
+        <v>46136</v>
+      </c>
+      <c r="B633" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C633" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D633" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E633" s="2"/>
+      <c r="F633" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G633" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H633" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I633" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J633" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K633" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L633" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M633" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N633" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O633" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P633" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q633" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R633" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S633" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T633" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U633" s="2"/>
+      <c r="V633" s="2"/>
+      <c r="W633" s="2"/>
+      <c r="X633" s="2"/>
+      <c r="Y633" s="2"/>
+      <c r="Z633" s="2"/>
+      <c r="AA633" s="2"/>
+      <c r="AB633" s="2"/>
+      <c r="AC633" s="2"/>
+      <c r="AD633" s="2"/>
+    </row>
+    <row r="634" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A634" s="5">
+        <v>46137</v>
+      </c>
+      <c r="B634" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C634" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D634" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E634" s="2"/>
+      <c r="F634" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G634" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H634" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I634" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J634" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K634" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L634" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M634" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N634" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O634" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P634" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q634" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R634" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S634" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T634" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U634" s="2"/>
+      <c r="V634" s="2"/>
+      <c r="W634" s="2"/>
+      <c r="X634" s="2"/>
+      <c r="Y634" s="2"/>
+      <c r="Z634" s="2"/>
+      <c r="AA634" s="2"/>
+      <c r="AB634" s="2"/>
+      <c r="AC634" s="2"/>
+      <c r="AD634" s="2"/>
+    </row>
+    <row r="635" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A635" s="5">
+        <v>46138</v>
+      </c>
+      <c r="B635" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C635" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D635" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E635" s="2"/>
+      <c r="F635" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G635" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H635" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I635" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J635" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K635" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L635" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M635" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N635" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O635" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P635" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q635" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R635" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S635" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T635" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U635" s="2"/>
+      <c r="V635" s="2"/>
+      <c r="W635" s="2"/>
+      <c r="X635" s="2"/>
+      <c r="Y635" s="2"/>
+      <c r="Z635" s="2"/>
+      <c r="AA635" s="2"/>
+      <c r="AB635" s="2"/>
+      <c r="AC635" s="2"/>
+      <c r="AD635" s="2"/>
+    </row>
+    <row r="636" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A636" s="5">
+        <v>46139</v>
+      </c>
+      <c r="B636" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C636" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D636" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E636" s="2"/>
+      <c r="F636" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G636" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H636" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I636" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J636" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K636" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L636" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M636" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N636" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O636" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P636" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q636" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R636" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S636" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T636" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U636" s="2"/>
+      <c r="V636" s="2"/>
+      <c r="W636" s="2"/>
+      <c r="X636" s="2"/>
+      <c r="Y636" s="2"/>
+      <c r="Z636" s="2"/>
+      <c r="AA636" s="2"/>
+      <c r="AB636" s="2"/>
+      <c r="AC636" s="2"/>
+      <c r="AD636" s="2"/>
+    </row>
+    <row r="637" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A637" s="5">
+        <v>46140</v>
+      </c>
+      <c r="B637" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C637" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D637" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E637" s="2"/>
+      <c r="F637" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G637" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H637" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I637" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J637" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K637" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L637" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M637" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N637" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O637" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P637" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q637" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R637" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S637" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T637" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U637" s="2"/>
+      <c r="V637" s="2"/>
+      <c r="W637" s="2"/>
+      <c r="X637" s="2"/>
+      <c r="Y637" s="2"/>
+      <c r="Z637" s="2"/>
+      <c r="AA637" s="2"/>
+      <c r="AB637" s="2"/>
+      <c r="AC637" s="2"/>
+      <c r="AD637" s="2"/>
+    </row>
+    <row r="638" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A638" s="5">
+        <v>46141</v>
+      </c>
+      <c r="B638" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C638" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D638" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E638" s="2"/>
+      <c r="F638" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G638" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H638" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I638" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J638" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K638" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L638" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M638" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N638" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O638" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P638" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q638" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R638" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S638" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T638" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U638" s="2"/>
+      <c r="V638" s="2"/>
+      <c r="W638" s="2"/>
+      <c r="X638" s="2"/>
+      <c r="Y638" s="2"/>
+      <c r="Z638" s="2"/>
+      <c r="AA638" s="2"/>
+      <c r="AB638" s="2"/>
+      <c r="AC638" s="2"/>
+      <c r="AD638" s="2"/>
+    </row>
+    <row r="639" spans="1:30" ht="13" x14ac:dyDescent="0.15">
+      <c r="A639" s="5">
+        <v>46142</v>
+      </c>
+      <c r="B639" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C639" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D639" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E639" s="2"/>
+      <c r="F639" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G639" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H639" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I639" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J639" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K639" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L639" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M639" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N639" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O639" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P639" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q639" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R639" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S639" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T639" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U639" s="2"/>
+      <c r="V639" s="2"/>
+      <c r="W639" s="2"/>
+      <c r="X639" s="2"/>
+      <c r="Y639" s="2"/>
+      <c r="Z639" s="2"/>
+      <c r="AA639" s="2"/>
+      <c r="AB639" s="2"/>
+      <c r="AC639" s="2"/>
+      <c r="AD639" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -40605,7 +42495,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:S612"/>
+  <dimension ref="A1:S639"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="2" max="2" width="11.6640625" customWidth="1"/>
@@ -75215,6 +77105,1545 @@
         <v>24</v>
       </c>
     </row>
+    <row r="613" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A613" s="5">
+        <v>46116</v>
+      </c>
+      <c r="B613" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C613" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D613" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E613" s="1"/>
+      <c r="F613" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G613" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H613" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I613" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J613" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K613" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L613" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M613" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N613" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O613" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P613" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q613" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R613" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S613" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="614" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A614" s="5">
+        <v>46117</v>
+      </c>
+      <c r="B614" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C614" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D614" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E614" s="1"/>
+      <c r="F614" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G614" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H614" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I614" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J614" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K614" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L614" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M614" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N614" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O614" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P614" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q614" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R614" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S614" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="615" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A615" s="5">
+        <v>46118</v>
+      </c>
+      <c r="B615" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C615" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D615" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E615" s="1"/>
+      <c r="F615" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G615" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H615" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I615" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J615" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K615" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L615" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M615" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N615" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O615" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P615" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q615" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R615" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S615" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="616" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A616" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B616" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C616" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D616" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E616" s="1"/>
+      <c r="F616" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G616" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H616" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I616" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J616" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K616" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L616" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M616" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N616" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O616" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P616" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q616" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R616" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S616" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="617" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A617" s="5">
+        <v>46120</v>
+      </c>
+      <c r="B617" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C617" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D617" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E617" s="1"/>
+      <c r="F617" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G617" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H617" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I617" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J617" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K617" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L617" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M617" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N617" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O617" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P617" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q617" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R617" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S617" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="618" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A618" s="5">
+        <v>46121</v>
+      </c>
+      <c r="B618" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C618" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D618" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E618" s="1"/>
+      <c r="F618" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G618" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H618" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I618" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J618" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K618" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L618" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M618" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N618" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O618" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P618" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q618" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R618" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S618" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="619" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A619" s="5">
+        <v>46122</v>
+      </c>
+      <c r="B619" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C619" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D619" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E619" s="1"/>
+      <c r="F619" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G619" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H619" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I619" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J619" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K619" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L619" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M619" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N619" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O619" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P619" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q619" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R619" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S619" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="620" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A620" s="5">
+        <v>46123</v>
+      </c>
+      <c r="B620" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C620" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D620" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E620" s="1"/>
+      <c r="F620" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G620" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H620" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I620" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J620" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K620" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L620" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M620" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N620" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O620" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P620" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q620" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R620" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S620" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="621" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A621" s="5">
+        <v>46124</v>
+      </c>
+      <c r="B621" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C621" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D621" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E621" s="1"/>
+      <c r="F621" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G621" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H621" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I621" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J621" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K621" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L621" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M621" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N621" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O621" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P621" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q621" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R621" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S621" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="622" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A622" s="5">
+        <v>46125</v>
+      </c>
+      <c r="B622" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C622" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D622" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E622" s="1"/>
+      <c r="F622" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G622" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H622" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I622" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J622" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K622" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L622" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M622" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N622" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O622" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P622" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q622" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R622" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S622" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="623" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A623" s="5">
+        <v>46126</v>
+      </c>
+      <c r="B623" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C623" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D623" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E623" s="1"/>
+      <c r="F623" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G623" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H623" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I623" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J623" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K623" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L623" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M623" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N623" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O623" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P623" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q623" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R623" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S623" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="624" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A624" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B624" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C624" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D624" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E624" s="1"/>
+      <c r="F624" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G624" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H624" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I624" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J624" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K624" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L624" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M624" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N624" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O624" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P624" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q624" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R624" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S624" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="625" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A625" s="5">
+        <v>46128</v>
+      </c>
+      <c r="B625" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C625" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D625" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E625" s="1"/>
+      <c r="F625" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G625" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H625" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I625" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J625" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K625" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L625" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M625" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N625" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O625" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P625" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q625" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R625" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S625" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="626" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A626" s="5">
+        <v>46129</v>
+      </c>
+      <c r="B626" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C626" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D626" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E626" s="1"/>
+      <c r="F626" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G626" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H626" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I626" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J626" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K626" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L626" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M626" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N626" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O626" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P626" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q626" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R626" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S626" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="627" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A627" s="5">
+        <v>46130</v>
+      </c>
+      <c r="B627" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C627" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D627" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E627" s="1"/>
+      <c r="F627" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G627" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H627" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I627" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J627" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K627" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L627" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M627" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N627" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O627" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P627" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q627" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R627" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S627" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="628" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A628" s="5">
+        <v>46131</v>
+      </c>
+      <c r="B628" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C628" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D628" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E628" s="1"/>
+      <c r="F628" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G628" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H628" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I628" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J628" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K628" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L628" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M628" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N628" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O628" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P628" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q628" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R628" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S628" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="629" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A629" s="5">
+        <v>46132</v>
+      </c>
+      <c r="B629" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C629" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D629" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E629" s="1"/>
+      <c r="F629" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G629" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H629" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I629" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J629" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K629" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L629" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M629" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N629" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O629" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P629" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q629" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R629" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S629" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="630" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A630" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B630" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C630" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D630" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E630" s="1"/>
+      <c r="F630" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G630" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H630" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I630" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J630" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K630" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L630" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M630" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N630" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O630" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P630" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q630" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R630" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S630" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="631" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A631" s="5">
+        <v>46134</v>
+      </c>
+      <c r="B631" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C631" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D631" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E631" s="1"/>
+      <c r="F631" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G631" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H631" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I631" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J631" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K631" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L631" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M631" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N631" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O631" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P631" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q631" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R631" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S631" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="632" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A632" s="5">
+        <v>46135</v>
+      </c>
+      <c r="B632" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C632" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D632" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E632" s="1"/>
+      <c r="F632" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G632" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H632" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I632" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J632" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K632" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L632" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M632" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N632" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O632" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P632" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q632" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R632" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S632" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="633" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A633" s="5">
+        <v>46136</v>
+      </c>
+      <c r="B633" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C633" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D633" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E633" s="1"/>
+      <c r="F633" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G633" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H633" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I633" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J633" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K633" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L633" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M633" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N633" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O633" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P633" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q633" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R633" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S633" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="634" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A634" s="5">
+        <v>46137</v>
+      </c>
+      <c r="B634" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C634" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D634" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E634" s="1"/>
+      <c r="F634" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G634" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H634" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I634" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J634" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K634" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L634" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M634" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N634" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O634" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P634" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q634" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R634" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S634" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="635" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A635" s="5">
+        <v>46138</v>
+      </c>
+      <c r="B635" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C635" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D635" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E635" s="1"/>
+      <c r="F635" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G635" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H635" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I635" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J635" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K635" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L635" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M635" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N635" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O635" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P635" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q635" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R635" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S635" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="636" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A636" s="5">
+        <v>46139</v>
+      </c>
+      <c r="B636" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C636" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D636" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E636" s="1"/>
+      <c r="F636" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G636" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H636" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I636" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J636" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K636" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L636" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M636" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N636" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O636" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P636" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q636" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R636" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S636" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="637" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A637" s="5">
+        <v>46140</v>
+      </c>
+      <c r="B637" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C637" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D637" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E637" s="1"/>
+      <c r="F637" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G637" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H637" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I637" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J637" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K637" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L637" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M637" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N637" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O637" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P637" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q637" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R637" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S637" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="638" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A638" s="5">
+        <v>46141</v>
+      </c>
+      <c r="B638" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C638" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D638" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E638" s="1"/>
+      <c r="F638" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G638" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H638" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I638" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J638" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K638" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L638" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M638" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N638" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O638" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P638" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q638" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R638" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S638" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="639" spans="1:19" ht="13" x14ac:dyDescent="0.15">
+      <c r="A639" s="5">
+        <v>46142</v>
+      </c>
+      <c r="B639" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C639" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D639" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E639" s="1"/>
+      <c r="F639" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G639" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H639" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I639" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J639" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K639" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L639" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M639" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N639" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O639" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P639" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q639" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R639" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S639" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>